<commit_message>
Update for Revision II
</commit_message>
<xml_diff>
--- a/docs/Results/Counties/Baden-Württemberg/pop_results_Landkreis_Alb-Donau-Kreis_CT_vs_Stroke.xlsx
+++ b/docs/Results/Counties/Baden-Württemberg/pop_results_Landkreis_Alb-Donau-Kreis_CT_vs_Stroke.xlsx
@@ -645,7 +645,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -661,7 +661,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -677,7 +677,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -693,7 +693,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -709,7 +709,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -725,7 +725,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -741,7 +741,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -757,7 +757,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -773,7 +773,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -789,7 +789,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -805,7 +805,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -821,7 +821,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Extended Stroke Hospitals</t>
+          <t>Stroke-Ready Hospitals</t>
         </is>
       </c>
       <c r="B25" t="n">

</xml_diff>